<commit_message>
Actualizacion del sistema para arrojar graficos de prediccion y estar listo para pruebas medicas
</commit_message>
<xml_diff>
--- a/ml/outputs/SavedModels/training_metrics_report.xlsx
+++ b/ml/outputs/SavedModels/training_metrics_report.xlsx
@@ -24,9 +24,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Comparacion_Modelos'!$A$1:$AN$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Particion_Datos'!$A$1:$K$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Hiperparametros'!$A$1:$E$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Variables_Relevantes'!$A$1:$F$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Variables_Relevantes'!$A$1:$F$32</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tiempos_Prediccion'!$A$1:$F$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Targets_Omitidos'!$A$1:$F$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Targets_Omitidos'!$A$1:$F$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Resumen'!$A$1:$L$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'CV_Detallado'!$A$1:$P$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Variables_Seleccionadas'!$A$1:$E$57</definedName>
@@ -461,11 +461,11 @@
     <col width="21" customWidth="1" min="9" max="9"/>
     <col width="21" customWidth="1" min="10" max="10"/>
     <col width="21" customWidth="1" min="11" max="11"/>
-    <col width="21" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
     <col width="21" customWidth="1" min="13" max="13"/>
     <col width="21" customWidth="1" min="14" max="14"/>
-    <col width="21" customWidth="1" min="15" max="15"/>
-    <col width="23" customWidth="1" min="16" max="16"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="21" customWidth="1" min="16" max="16"/>
     <col width="22" customWidth="1" min="17" max="17"/>
     <col width="21" customWidth="1" min="18" max="18"/>
     <col width="26" customWidth="1" min="19" max="19"/>
@@ -727,41 +727,41 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>0.8457639522212423</v>
+        <v>0.6981796410006491</v>
       </c>
       <c r="I2" t="n">
-        <v>0.4409606861810243</v>
+        <v>0.7218428110993059</v>
       </c>
       <c r="J2" t="n">
-        <v>0.1347830351222189</v>
+        <v>0.05531678862705329</v>
       </c>
       <c r="K2" t="n">
-        <v>0.8666666666666667</v>
+        <v>0.6875</v>
       </c>
       <c r="L2" t="n">
-        <v>0.8571428571428571</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="M2" t="n">
-        <v>0.8333333333333333</v>
+        <v>0.7083333333333333</v>
       </c>
       <c r="N2" t="n">
-        <v>0.8388888888888888</v>
+        <v>0.6892857142857143</v>
       </c>
       <c r="O2" t="n">
-        <v>0.9696969696969697</v>
+        <v>0.9022727272727273</v>
       </c>
       <c r="P2" t="n">
-        <v>0.8125783774660579</v>
+        <v>0.620704416451776</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.806896551724138</v>
+        <v>0.6164383561643836</v>
       </c>
       <c r="R2" t="n">
-        <v>0.8333333333333333</v>
+        <v>0.7083333333333333</v>
       </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr"/>
@@ -782,7 +782,7 @@
       <c r="AI2" t="inlineStr"/>
       <c r="AJ2" t="inlineStr"/>
       <c r="AK2" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="AL2" t="n">
         <v>14</v>
@@ -829,37 +829,37 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>0.2349718933155498</v>
+        <v>0.4587347149150859</v>
       </c>
       <c r="I3" t="n">
-        <v>0.2202617942239165</v>
+        <v>0.3373921080737929</v>
       </c>
       <c r="J3" t="n">
-        <v>0.01898143560601258</v>
+        <v>0.09337965042254821</v>
       </c>
       <c r="K3" t="n">
-        <v>0.2916666666666666</v>
+        <v>0.4583333333333333</v>
       </c>
       <c r="L3" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.5</v>
       </c>
       <c r="M3" t="n">
-        <v>0.2708333333333333</v>
+        <v>0.4791666666666666</v>
       </c>
       <c r="N3" t="n">
-        <v>0.2714285714285715</v>
+        <v>0.4595238095238094</v>
       </c>
       <c r="O3" t="n">
-        <v>0.5892045454545454</v>
+        <v>0.7270833333333333</v>
       </c>
       <c r="P3" t="n">
-        <v>0.03522524587835815</v>
+        <v>0.3311173112565667</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.03448275862068972</v>
+        <v>0.3241379310344827</v>
       </c>
       <c r="R3" t="n">
-        <v>0.2708333333333333</v>
+        <v>0.4791666666666666</v>
       </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr"/>
@@ -880,7 +880,7 @@
       <c r="AI3" t="inlineStr"/>
       <c r="AJ3" t="inlineStr"/>
       <c r="AK3" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="AL3" t="n">
         <v>14</v>
@@ -927,37 +927,37 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>0.8450063764636665</v>
+        <v>0.7818678099135439</v>
       </c>
       <c r="I4" t="n">
-        <v>0.5149901422055275</v>
+        <v>0.6610063270859833</v>
       </c>
       <c r="J4" t="n">
-        <v>0.06428660593185651</v>
+        <v>0.08991087054204888</v>
       </c>
       <c r="K4" t="n">
-        <v>0.8666666666666667</v>
+        <v>0.8375</v>
       </c>
       <c r="L4" t="n">
-        <v>0.8571428571428571</v>
+        <v>0.7857142857142857</v>
       </c>
       <c r="M4" t="n">
-        <v>0.8333333333333333</v>
+        <v>0.7916666666666666</v>
       </c>
       <c r="N4" t="n">
-        <v>0.8388888888888888</v>
+        <v>0.8041666666666667</v>
       </c>
       <c r="O4" t="n">
-        <v>0.9621212121212122</v>
+        <v>0.9170454545454545</v>
       </c>
       <c r="P4" t="n">
-        <v>0.8125783774660579</v>
+        <v>0.7153467767436237</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.806896551724138</v>
+        <v>0.710344827586207</v>
       </c>
       <c r="R4" t="n">
-        <v>0.8333333333333333</v>
+        <v>0.7916666666666666</v>
       </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr"/>
@@ -978,7 +978,7 @@
       <c r="AI4" t="inlineStr"/>
       <c r="AJ4" t="inlineStr"/>
       <c r="AK4" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="AL4" t="n">
         <v>14</v>
@@ -1025,37 +1025,37 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>0.7757197035990275</v>
+        <v>0.765833407166251</v>
       </c>
       <c r="I5" t="n">
-        <v>0.4847565827692084</v>
+        <v>0.7660041561011978</v>
       </c>
       <c r="J5" t="n">
-        <v>0.1742643403567872</v>
+        <v>0.123166892445981</v>
       </c>
       <c r="K5" t="n">
-        <v>0.8333333333333333</v>
+        <v>0.8541666666666666</v>
       </c>
       <c r="L5" t="n">
         <v>0.7857142857142857</v>
       </c>
       <c r="M5" t="n">
-        <v>0.7708333333333333</v>
+        <v>0.7708333333333334</v>
       </c>
       <c r="N5" t="n">
-        <v>0.7809523809523808</v>
+        <v>0.7535714285714286</v>
       </c>
       <c r="O5" t="n">
-        <v>0.928219696969697</v>
+        <v>0.8679924242424242</v>
       </c>
       <c r="P5" t="n">
-        <v>0.725640065094178</v>
+        <v>0.7363908738684537</v>
       </c>
       <c r="Q5" t="n">
         <v>0.710344827586207</v>
       </c>
       <c r="R5" t="n">
-        <v>0.7708333333333333</v>
+        <v>0.7708333333333334</v>
       </c>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr"/>
@@ -1076,7 +1076,7 @@
       <c r="AI5" t="inlineStr"/>
       <c r="AJ5" t="inlineStr"/>
       <c r="AK5" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="AL5" t="n">
         <v>14</v>
@@ -1123,37 +1123,37 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>0.6318798041476351</v>
+        <v>0.697485619489256</v>
       </c>
       <c r="I6" t="n">
-        <v>0.6006481598807721</v>
+        <v>0.7844813451002542</v>
       </c>
       <c r="J6" t="n">
-        <v>0.1012698009245711</v>
+        <v>0.09665484830832617</v>
       </c>
       <c r="K6" t="n">
-        <v>0.6845238095238095</v>
+        <v>0.7125</v>
       </c>
       <c r="L6" t="n">
-        <v>0.6428571428571429</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="M6" t="n">
-        <v>0.625</v>
+        <v>0.7083333333333333</v>
       </c>
       <c r="N6" t="n">
-        <v>0.6246753246753247</v>
+        <v>0.6952380952380952</v>
       </c>
       <c r="O6" t="n">
-        <v>0.9571969696969698</v>
+        <v>0.8768939393939394</v>
       </c>
       <c r="P6" t="n">
-        <v>0.5371352022540757</v>
+        <v>0.6250602903585061</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.5138888888888888</v>
+        <v>0.6164383561643836</v>
       </c>
       <c r="R6" t="n">
-        <v>0.625</v>
+        <v>0.7083333333333333</v>
       </c>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr"/>
@@ -1174,7 +1174,7 @@
       <c r="AI6" t="inlineStr"/>
       <c r="AJ6" t="inlineStr"/>
       <c r="AK6" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="AL6" t="n">
         <v>14</v>
@@ -1217,41 +1217,41 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>0.7882205481192686</v>
+        <v>0.6952507710044076</v>
       </c>
       <c r="I7" t="n">
-        <v>0.3779754761237398</v>
+        <v>0.4876148990953708</v>
       </c>
       <c r="J7" t="n">
-        <v>0.1170607850444378</v>
+        <v>0.09148832674172856</v>
       </c>
       <c r="K7" t="n">
-        <v>0.8166666666666667</v>
+        <v>0.7125</v>
       </c>
       <c r="L7" t="n">
-        <v>0.7857142857142857</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="M7" t="n">
-        <v>0.8125</v>
+        <v>0.7083333333333333</v>
       </c>
       <c r="N7" t="n">
-        <v>0.8095238095238095</v>
+        <v>0.6952380952380952</v>
       </c>
       <c r="O7" t="n">
-        <v>0.9223484848484849</v>
+        <v>0.8545454545454546</v>
       </c>
       <c r="P7" t="n">
-        <v>0.7172584367887189</v>
+        <v>0.6250602903585061</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.7123287671232876</v>
+        <v>0.6164383561643836</v>
       </c>
       <c r="R7" t="n">
-        <v>0.8125</v>
+        <v>0.7083333333333333</v>
       </c>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr"/>
@@ -1272,7 +1272,7 @@
       <c r="AI7" t="inlineStr"/>
       <c r="AJ7" t="inlineStr"/>
       <c r="AK7" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="AL7" t="n">
         <v>14</v>
@@ -1319,37 +1319,37 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>0.1685981171023997</v>
+        <v>0.4630659384038094</v>
       </c>
       <c r="I8" t="n">
-        <v>0.3449742684747331</v>
+        <v>0.4298335287550849</v>
       </c>
       <c r="J8" t="n">
-        <v>0.1018044308232209</v>
+        <v>0.1437952014675728</v>
       </c>
       <c r="K8" t="n">
-        <v>0.125</v>
+        <v>0.5166666666666666</v>
       </c>
       <c r="L8" t="n">
-        <v>0.2142857142857143</v>
+        <v>0.5</v>
       </c>
       <c r="M8" t="n">
-        <v>0.2083333333333333</v>
+        <v>0.4791666666666666</v>
       </c>
       <c r="N8" t="n">
-        <v>0.1555555555555556</v>
+        <v>0.492063492063492</v>
       </c>
       <c r="O8" t="n">
-        <v>0.6797348484848486</v>
+        <v>0.6984848484848485</v>
       </c>
       <c r="P8" t="n">
-        <v>-0.05244954158765781</v>
+        <v>0.3310423554409472</v>
       </c>
       <c r="Q8" t="n">
-        <v>-0.04761904761904767</v>
+        <v>0.3287671232876712</v>
       </c>
       <c r="R8" t="n">
-        <v>0.2083333333333333</v>
+        <v>0.4791666666666666</v>
       </c>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr"/>
@@ -1370,7 +1370,7 @@
       <c r="AI8" t="inlineStr"/>
       <c r="AJ8" t="inlineStr"/>
       <c r="AK8" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="AL8" t="n">
         <v>14</v>
@@ -1417,37 +1417,37 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>0.4012302832645255</v>
+        <v>0.6078522056552473</v>
       </c>
       <c r="I9" t="n">
-        <v>0.2991408552503636</v>
+        <v>0.3892946234036278</v>
       </c>
       <c r="J9" t="n">
-        <v>0.03917440305639606</v>
+        <v>0.1297625288014696</v>
       </c>
       <c r="K9" t="n">
-        <v>0.5333333333333333</v>
+        <v>0.5625</v>
       </c>
       <c r="L9" t="n">
-        <v>0.4285714285714285</v>
+        <v>0.6428571428571429</v>
       </c>
       <c r="M9" t="n">
-        <v>0.4166666666666666</v>
+        <v>0.625</v>
       </c>
       <c r="N9" t="n">
-        <v>0.4305555555555555</v>
+        <v>0.5785714285714285</v>
       </c>
       <c r="O9" t="n">
-        <v>0.7867424242424244</v>
+        <v>0.8054924242424242</v>
       </c>
       <c r="P9" t="n">
-        <v>0.2270931823214638</v>
+        <v>0.5362069469915925</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.2222222222222221</v>
+        <v>0.5172413793103449</v>
       </c>
       <c r="R9" t="n">
-        <v>0.4166666666666666</v>
+        <v>0.625</v>
       </c>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr"/>
@@ -1468,7 +1468,7 @@
       <c r="AI9" t="inlineStr"/>
       <c r="AJ9" t="inlineStr"/>
       <c r="AK9" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="AL9" t="n">
         <v>14</v>
@@ -1515,37 +1515,37 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>0.1558815958815959</v>
+        <v>0.3363095238095238</v>
       </c>
       <c r="I10" t="n">
-        <v>0.3395696413877416</v>
+        <v>0.3533464268161774</v>
       </c>
       <c r="J10" t="n">
-        <v>0.2028798516360231</v>
+        <v>0.06083822977673526</v>
       </c>
       <c r="K10" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="N10" t="n">
         <v>0.2857142857142857</v>
       </c>
-      <c r="L10" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="M10" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="N10" t="n">
-        <v>0.3333333333333333</v>
-      </c>
       <c r="O10" t="n">
-        <v>0.4571428571428571</v>
+        <v>0.625</v>
       </c>
       <c r="P10" t="n">
-        <v>-0.3142857142857143</v>
+        <v>0</v>
       </c>
       <c r="Q10" t="n">
-        <v>-0.2972972972972974</v>
+        <v>0</v>
       </c>
       <c r="R10" t="n">
-        <v>0.3428571428571429</v>
+        <v>0.5</v>
       </c>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr"/>
@@ -1566,7 +1566,7 @@
       <c r="AI10" t="inlineStr"/>
       <c r="AJ10" t="inlineStr"/>
       <c r="AK10" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="AL10" t="n">
         <v>12</v>
@@ -1613,37 +1613,37 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>0.4068453292333867</v>
+        <v>0.3951456538798342</v>
       </c>
       <c r="I11" t="n">
-        <v>0.3737211663951442</v>
+        <v>0.4028869136588666</v>
       </c>
       <c r="J11" t="n">
-        <v>0.2659761594942385</v>
+        <v>0.139140091547024</v>
       </c>
       <c r="K11" t="n">
         <v>0.5</v>
       </c>
       <c r="L11" t="n">
-        <v>0.5833333333333334</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="M11" t="n">
-        <v>0.4</v>
+        <v>0.25</v>
       </c>
       <c r="N11" t="n">
-        <v>0.4444444444444444</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="O11" t="n">
-        <v>0.5428571428571429</v>
+        <v>0.375</v>
       </c>
       <c r="P11" t="n">
-        <v>0.1195228609334394</v>
+        <v>0.158113883008419</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.1176470588235294</v>
+        <v>0.1428571428571429</v>
       </c>
       <c r="R11" t="n">
-        <v>0.5571428571428572</v>
+        <v>0.5625</v>
       </c>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr"/>
@@ -1664,7 +1664,7 @@
       <c r="AI11" t="inlineStr"/>
       <c r="AJ11" t="inlineStr"/>
       <c r="AK11" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="AL11" t="n">
         <v>12</v>
@@ -1702,46 +1702,46 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
       <c r="H12" t="n">
-        <v>0.2588679924122655</v>
+        <v>0.6381352851875146</v>
       </c>
       <c r="I12" t="n">
-        <v>0.268291384678758</v>
+        <v>0.4966328465756196</v>
       </c>
       <c r="J12" t="n">
-        <v>0.1520907575590468</v>
+        <v>0.02484635610019794</v>
       </c>
       <c r="K12" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.6</v>
       </c>
       <c r="L12" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="M12" t="n">
-        <v>0.2</v>
+        <v>0.75</v>
       </c>
       <c r="N12" t="n">
-        <v>0.25</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="O12" t="n">
-        <v>0.4571428571428572</v>
+        <v>0.625</v>
       </c>
       <c r="P12" t="n">
-        <v>-0.09759000729485331</v>
+        <v>0.4780914437337574</v>
       </c>
       <c r="Q12" t="n">
-        <v>-0.09090909090909083</v>
+        <v>0.4705882352941176</v>
       </c>
       <c r="R12" t="n">
-        <v>0.4571428571428572</v>
+        <v>0.75</v>
       </c>
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr"/>
@@ -1762,7 +1762,7 @@
       <c r="AI12" t="inlineStr"/>
       <c r="AJ12" t="inlineStr"/>
       <c r="AK12" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="AL12" t="n">
         <v>12</v>
@@ -1809,37 +1809,37 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>0.2342774069901791</v>
+        <v>0.4833333333333332</v>
       </c>
       <c r="I13" t="n">
-        <v>0.2893178792758322</v>
+        <v>0.3079790595926196</v>
       </c>
       <c r="J13" t="n">
-        <v>0.1234649722951741</v>
+        <v>0.05287581298375235</v>
       </c>
       <c r="K13" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.5</v>
       </c>
       <c r="L13" t="n">
-        <v>0.4166666666666667</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="M13" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="N13" t="n">
-        <v>0.3636363636363636</v>
+        <v>0.5</v>
       </c>
       <c r="O13" t="n">
-        <v>0.4571428571428572</v>
+        <v>0.5</v>
       </c>
       <c r="P13" t="n">
-        <v>-0.1690308509457033</v>
+        <v>0.25</v>
       </c>
       <c r="Q13" t="n">
-        <v>-0.1666666666666667</v>
+        <v>0.25</v>
       </c>
       <c r="R13" t="n">
-        <v>0.4142857142857143</v>
+        <v>0.625</v>
       </c>
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr"/>
@@ -1860,7 +1860,7 @@
       <c r="AI13" t="inlineStr"/>
       <c r="AJ13" t="inlineStr"/>
       <c r="AK13" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="AL13" t="n">
         <v>12</v>
@@ -1907,37 +1907,37 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>0.2428488355616077</v>
+        <v>0.333125</v>
       </c>
       <c r="I14" t="n">
-        <v>0.3249109438725725</v>
+        <v>0.3297968269867557</v>
       </c>
       <c r="J14" t="n">
-        <v>0.1121431800978097</v>
+        <v>0.08560378777775565</v>
       </c>
       <c r="K14" t="n">
         <v>0.3333333333333333</v>
       </c>
       <c r="L14" t="n">
-        <v>0.4166666666666667</v>
+        <v>0.5</v>
       </c>
       <c r="M14" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N14" t="n">
         <v>0.4</v>
       </c>
-      <c r="N14" t="n">
-        <v>0.3636363636363636</v>
-      </c>
       <c r="O14" t="n">
-        <v>0.5428571428571429</v>
+        <v>0.53125</v>
       </c>
       <c r="P14" t="n">
-        <v>-0.1690308509457033</v>
+        <v>0</v>
       </c>
       <c r="Q14" t="n">
-        <v>-0.1666666666666667</v>
+        <v>0</v>
       </c>
       <c r="R14" t="n">
-        <v>0.4142857142857143</v>
+        <v>0.5</v>
       </c>
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr"/>
@@ -1958,7 +1958,7 @@
       <c r="AI14" t="inlineStr"/>
       <c r="AJ14" t="inlineStr"/>
       <c r="AK14" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="AL14" t="n">
         <v>12</v>
@@ -1996,7 +1996,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -2005,37 +2005,37 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>0.4503979176851455</v>
+        <v>0.314375</v>
       </c>
       <c r="I15" t="n">
-        <v>0.3585353840029146</v>
+        <v>0.4210658128593686</v>
       </c>
       <c r="J15" t="n">
-        <v>0.1751465202381481</v>
+        <v>0.04870799251698639</v>
       </c>
       <c r="K15" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L15" t="n">
         <v>0.5</v>
       </c>
-      <c r="L15" t="n">
-        <v>0.5833333333333334</v>
-      </c>
       <c r="M15" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="N15" t="n">
-        <v>0.5454545454545454</v>
+        <v>0.4</v>
       </c>
       <c r="O15" t="n">
-        <v>0.5714285714285714</v>
+        <v>0.34375</v>
       </c>
       <c r="P15" t="n">
-        <v>0.1690308509457033</v>
+        <v>0</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.1666666666666666</v>
+        <v>0</v>
       </c>
       <c r="R15" t="n">
-        <v>0.5857142857142856</v>
+        <v>0.5</v>
       </c>
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr"/>
@@ -2056,7 +2056,7 @@
       <c r="AI15" t="inlineStr"/>
       <c r="AJ15" t="inlineStr"/>
       <c r="AK15" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="AL15" t="n">
         <v>12</v>
@@ -2103,37 +2103,37 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>0.3626254826254826</v>
+        <v>0.333125</v>
       </c>
       <c r="I16" t="n">
-        <v>0.304661058469108</v>
+        <v>0.349127803328164</v>
       </c>
       <c r="J16" t="n">
-        <v>0.1628098406182071</v>
+        <v>0.02539952931696224</v>
       </c>
       <c r="K16" t="n">
-        <v>0.4285714285714285</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="L16" t="n">
         <v>0.5</v>
       </c>
       <c r="M16" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="N16" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0.53125</v>
+      </c>
+      <c r="P16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>0</v>
+      </c>
+      <c r="R16" t="n">
         <v>0.5</v>
-      </c>
-      <c r="O16" t="n">
-        <v>0.5142857142857142</v>
-      </c>
-      <c r="P16" t="n">
-        <v>0.02857142857142857</v>
-      </c>
-      <c r="Q16" t="n">
-        <v>0.02702702702702697</v>
-      </c>
-      <c r="R16" t="n">
-        <v>0.5142857142857142</v>
       </c>
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr"/>
@@ -2154,7 +2154,7 @@
       <c r="AI16" t="inlineStr"/>
       <c r="AJ16" t="inlineStr"/>
       <c r="AK16" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="AL16" t="n">
         <v>12</v>
@@ -2201,37 +2201,37 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>0.4446836319708597</v>
+        <v>0.1036336580776756</v>
       </c>
       <c r="I17" t="n">
-        <v>0.371507974042635</v>
+        <v>0.3782862730182292</v>
       </c>
       <c r="J17" t="n">
-        <v>0.2223646918967358</v>
+        <v>0.08014245821669674</v>
       </c>
       <c r="K17" t="n">
-        <v>0.5</v>
+        <v>0.1666666666666667</v>
       </c>
       <c r="L17" t="n">
-        <v>0.5833333333333334</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="M17" t="n">
-        <v>0.6</v>
+        <v>0.25</v>
       </c>
       <c r="N17" t="n">
-        <v>0.5454545454545454</v>
+        <v>0.2</v>
       </c>
       <c r="O17" t="n">
-        <v>0.5142857142857143</v>
+        <v>0.375</v>
       </c>
       <c r="P17" t="n">
-        <v>0.1690308509457033</v>
+        <v>-0.3535533905932738</v>
       </c>
       <c r="Q17" t="n">
-        <v>0.1666666666666666</v>
+        <v>-0.3333333333333333</v>
       </c>
       <c r="R17" t="n">
-        <v>0.5857142857142856</v>
+        <v>0.3125</v>
       </c>
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr"/>
@@ -2252,7 +2252,7 @@
       <c r="AI17" t="inlineStr"/>
       <c r="AJ17" t="inlineStr"/>
       <c r="AK17" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="AL17" t="n">
         <v>12</v>
@@ -2420,10 +2420,10 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E6" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.5833333333333334</v>
       </c>
     </row>
     <row r="7">
@@ -2443,10 +2443,10 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E7" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.4166666666666667</v>
       </c>
     </row>
   </sheetData>
@@ -2558,7 +2558,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="6">
@@ -2627,7 +2627,7 @@
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="19" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
     <col width="48" customWidth="1" min="9" max="9"/>
     <col width="45" customWidth="1" min="10" max="10"/>
     <col width="48" customWidth="1" min="11" max="11"/>
@@ -2702,7 +2702,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D2" t="n">
         <v>14</v>
@@ -2711,13 +2711,13 @@
         <v>15</v>
       </c>
       <c r="F2" t="n">
-        <v>69.79166666666666</v>
+        <v>69.47368421052632</v>
       </c>
       <c r="G2" t="n">
-        <v>14.58333333333333</v>
+        <v>14.73684210526316</v>
       </c>
       <c r="H2" t="n">
-        <v>15.625</v>
+        <v>15.78947368421053</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -2747,7 +2747,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D3" t="n">
         <v>12</v>
@@ -2756,13 +2756,13 @@
         <v>12</v>
       </c>
       <c r="F3" t="n">
-        <v>69.62025316455697</v>
+        <v>69.23076923076923</v>
       </c>
       <c r="G3" t="n">
-        <v>15.18987341772152</v>
+        <v>15.38461538461539</v>
       </c>
       <c r="H3" t="n">
-        <v>15.18987341772152</v>
+        <v>15.38461538461539</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -3273,15 +3273,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F61"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3324,21 +3324,23 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>categorical__FEV1_80% or above</t>
+          <t>FEV1</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.1199756041169166</v>
-      </c>
-      <c r="E2" t="inlineStr"/>
+        <v>0.4666666666666666</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.09428090415820629</v>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>feature_importance</t>
+          <t>permutation_importance</t>
         </is>
       </c>
     </row>
@@ -3350,21 +3352,23 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>categorical__FEV1_&lt;30%</t>
+          <t>Location</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.08132804930210109</v>
-      </c>
-      <c r="E3" t="inlineStr"/>
+        <v>0.0666666666666666</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.0544331053951817</v>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>feature_importance</t>
+          <t>permutation_importance</t>
         </is>
       </c>
     </row>
@@ -3376,21 +3380,23 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>categorical__FEV1_&gt;80%</t>
+          <t>PackHistory</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.0673741996288299</v>
-      </c>
-      <c r="E4" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>feature_importance</t>
+          <t>permutation_importance</t>
         </is>
       </c>
     </row>
@@ -3402,21 +3408,23 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>categorical__Heart Rate_Higher</t>
+          <t>MWT1Best</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.0567531324923038</v>
-      </c>
-      <c r="E5" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>feature_importance</t>
+          <t>permutation_importance</t>
         </is>
       </c>
     </row>
@@ -3428,21 +3436,23 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>numeric__CAT</t>
+          <t>MWT1</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.0541489459574222</v>
-      </c>
-      <c r="E6" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>feature_importance</t>
+          <t>permutation_importance</t>
         </is>
       </c>
     </row>
@@ -3454,21 +3464,23 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>categorical__FEV1_50-79%</t>
+          <t>FVC</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.0507759228348732</v>
-      </c>
-      <c r="E7" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>feature_importance</t>
+          <t>permutation_importance</t>
         </is>
       </c>
     </row>
@@ -3480,21 +3492,23 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>categorical__FEV1_30-49%</t>
+          <t>Genero Sexo</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.0414461530745029</v>
-      </c>
-      <c r="E8" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>feature_importance</t>
+          <t>permutation_importance</t>
         </is>
       </c>
     </row>
@@ -3506,21 +3520,23 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>categorical__Temperature_High</t>
+          <t>HAD</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.0311631727963686</v>
-      </c>
-      <c r="E9" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>feature_importance</t>
+          <t>permutation_importance</t>
         </is>
       </c>
     </row>
@@ -3532,21 +3548,23 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>numeric__FEV1PRED</t>
+          <t>smoking</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.0294187422841787</v>
-      </c>
-      <c r="E10" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>feature_importance</t>
+          <t>permutation_importance</t>
         </is>
       </c>
     </row>
@@ -3558,21 +3576,23 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>numeric__MWT1</t>
+          <t>FVCPRED</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.0250429809093475</v>
-      </c>
-      <c r="E11" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>feature_importance</t>
+          <t>permutation_importance</t>
         </is>
       </c>
     </row>
@@ -3584,21 +3604,23 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>numeric__mMRC</t>
+          <t>CAT</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.0244621615856885</v>
-      </c>
-      <c r="E12" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>feature_importance</t>
+          <t>permutation_importance</t>
         </is>
       </c>
     </row>
@@ -3610,21 +3632,23 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>numeric__HAD</t>
+          <t>Respiratory Rate</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.0234976802021265</v>
-      </c>
-      <c r="E13" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>feature_importance</t>
+          <t>permutation_importance</t>
         </is>
       </c>
     </row>
@@ -3636,21 +3660,23 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>numeric__FVCPRED</t>
+          <t>Heart Rate</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.0230501890182495</v>
-      </c>
-      <c r="E14" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>feature_importance</t>
+          <t>permutation_importance</t>
         </is>
       </c>
     </row>
@@ -3662,21 +3688,23 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>numeric__SGRQ</t>
+          <t>mMRC</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.0218830779194831</v>
-      </c>
-      <c r="E15" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>feature_importance</t>
+          <t>permutation_importance</t>
         </is>
       </c>
     </row>
@@ -3688,21 +3716,23 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>numeric__Respiratory Rate</t>
+          <t>FEV1PRED</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.0212205611169338</v>
-      </c>
-      <c r="E16" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>feature_importance</t>
+          <t>permutation_importance</t>
         </is>
       </c>
     </row>
@@ -3714,21 +3744,23 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>categorical__status of smoking_No</t>
+          <t>OCUPACION</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.0211033057421445</v>
-      </c>
-      <c r="E17" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>feature_importance</t>
+          <t>permutation_importance</t>
         </is>
       </c>
     </row>
@@ -3740,21 +3772,23 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>categorical__Blood pressure_Higher</t>
+          <t>Altura_MSNM</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.0184729397296905</v>
-      </c>
-      <c r="E18" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>feature_importance</t>
+          <t>permutation_importance</t>
         </is>
       </c>
     </row>
@@ -3766,21 +3800,23 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>categorical__BMI,kg/m2 (IMC)_21&lt;BMI&lt;25</t>
+          <t>PESO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.0175559520721435</v>
-      </c>
-      <c r="E19" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>feature_importance</t>
+          <t>permutation_importance</t>
         </is>
       </c>
     </row>
@@ -3792,21 +3828,23 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>numeric__FVC</t>
+          <t>AtrialFib</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.015944005921483</v>
-      </c>
-      <c r="E20" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>feature_importance</t>
+          <t>permutation_importance</t>
         </is>
       </c>
     </row>
@@ -3818,21 +3856,23 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>categorical__Sputum_Purlent</t>
+          <t>DISCAPACIDAD</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.0155669637024402</v>
-      </c>
-      <c r="E21" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>feature_importance</t>
+          <t>permutation_importance</t>
         </is>
       </c>
     </row>
@@ -3844,21 +3884,23 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>categorical__status of smoking_Nunca</t>
+          <t>TIPODISCAPAC</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.0154470186680555</v>
-      </c>
-      <c r="E22" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>feature_importance</t>
+          <t>permutation_importance</t>
         </is>
       </c>
     </row>
@@ -3870,21 +3912,23 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>numeric__Altura_MSNM</t>
+          <t>MWT2</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.0140527449548244</v>
-      </c>
-      <c r="E23" t="inlineStr"/>
+        <v>-0.0222222222222222</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0.0314269680527354</v>
+      </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>feature_importance</t>
+          <t>permutation_importance</t>
         </is>
       </c>
     </row>
@@ -3896,21 +3940,23 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>numeric__MWT2</t>
+          <t>SGRQ</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.0139593761414289</v>
-      </c>
-      <c r="E24" t="inlineStr"/>
+        <v>-0.0222222222222222</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0.0314269680527354</v>
+      </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>feature_importance</t>
+          <t>permutation_importance</t>
         </is>
       </c>
     </row>
@@ -3922,21 +3968,23 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>categorical__FEV1_29% or less</t>
+          <t>Oxygen Saturation</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.013819370418787</v>
-      </c>
-      <c r="E25" t="inlineStr"/>
+        <v>-0.0222222222222222</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0.0314269680527354</v>
+      </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>feature_importance</t>
+          <t>permutation_importance</t>
         </is>
       </c>
     </row>
@@ -3948,21 +3996,23 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>numeric__MWT1Best</t>
+          <t>Temperature</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0.0128895482048392</v>
-      </c>
-      <c r="E26" t="inlineStr"/>
+        <v>-0.0222222222222222</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.0314269680527354</v>
+      </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>feature_importance</t>
+          <t>permutation_importance</t>
         </is>
       </c>
     </row>
@@ -3974,21 +4024,23 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>categorical__Temperature_Normal</t>
+          <t>Blood pressure</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0.0128887146711349</v>
-      </c>
-      <c r="E27" t="inlineStr"/>
+        <v>-0.0222222222222222</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.0314269680527354</v>
+      </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>feature_importance</t>
+          <t>permutation_importance</t>
         </is>
       </c>
     </row>
@@ -4000,21 +4052,23 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>categorical__Blood pressure_Elevate</t>
+          <t>EDAD</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0.0123217301443219</v>
-      </c>
-      <c r="E28" t="inlineStr"/>
+        <v>-0.0444444444444445</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0.0314269680527354</v>
+      </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>feature_importance</t>
+          <t>permutation_importance</t>
         </is>
       </c>
     </row>
@@ -4026,21 +4080,23 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>numeric__PackHistory</t>
+          <t>status of smoking</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>0.0117862969636917</v>
-      </c>
-      <c r="E29" t="inlineStr"/>
+        <v>-0.0444444444444445</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0.0314269680527354</v>
+      </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>feature_importance</t>
+          <t>permutation_importance</t>
         </is>
       </c>
     </row>
@@ -4052,21 +4108,23 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>numeric__TALLA(altura ó Height/m)</t>
+          <t>Sputum</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>0.0113291535526514</v>
-      </c>
-      <c r="E30" t="inlineStr"/>
+        <v>-0.0444444444444445</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0.0314269680527354</v>
+      </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>feature_importance</t>
+          <t>permutation_importance</t>
         </is>
       </c>
     </row>
@@ -4078,21 +4136,23 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>categorical__Temperature_Higher</t>
+          <t>BMI,kg/m2 (IMC)</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>0.010326930321753</v>
-      </c>
-      <c r="E31" t="inlineStr"/>
+        <v>-0.0444444444444445</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0.0314269680527354</v>
+      </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>feature_importance</t>
+          <t>permutation_importance</t>
         </is>
       </c>
     </row>
@@ -4104,780 +4164,22 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>categorical__Heart Rate_Lower</t>
-        </is>
-      </c>
-      <c r="D32" t="n">
-        <v>1.037911548280755</v>
-      </c>
-      <c r="E32" t="inlineStr"/>
+          <t>No disponible</t>
+        </is>
+      </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>absolute_coefficient</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>history_of_heart_failure</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>LogisticRegression</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>categorical__status of smoking_No</t>
-        </is>
-      </c>
-      <c r="D33" t="n">
-        <v>0.9061170754524702</v>
-      </c>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>absolute_coefficient</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>history_of_heart_failure</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>LogisticRegression</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>categorical__Sputum_purlent</t>
-        </is>
-      </c>
-      <c r="D34" t="n">
-        <v>0.8636160187787837</v>
-      </c>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>absolute_coefficient</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>history_of_heart_failure</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>LogisticRegression</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>categorical__Blood pressure_Normal</t>
-        </is>
-      </c>
-      <c r="D35" t="n">
-        <v>0.7253663134530901</v>
-      </c>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>absolute_coefficient</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>history_of_heart_failure</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>LogisticRegression</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>categorical__Heart Rate_84</t>
-        </is>
-      </c>
-      <c r="D36" t="n">
-        <v>0.7235635417984401</v>
-      </c>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>absolute_coefficient</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>history_of_heart_failure</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>LogisticRegression</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>categorical__Blood pressure_Crisis</t>
-        </is>
-      </c>
-      <c r="D37" t="n">
-        <v>0.7219260427438986</v>
-      </c>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>absolute_coefficient</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>history_of_heart_failure</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>LogisticRegression</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>categorical__Heart Rate_Normal</t>
-        </is>
-      </c>
-      <c r="D38" t="n">
-        <v>0.66807228645787</v>
-      </c>
-      <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>absolute_coefficient</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>history_of_heart_failure</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>LogisticRegression</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>categorical__Blood pressure_Stage 2</t>
-        </is>
-      </c>
-      <c r="D39" t="n">
-        <v>0.6323483796291816</v>
-      </c>
-      <c r="E39" t="inlineStr"/>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>absolute_coefficient</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>history_of_heart_failure</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>LogisticRegression</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>categorical__Heart Rate_69</t>
-        </is>
-      </c>
-      <c r="D40" t="n">
-        <v>0.609276064439972</v>
-      </c>
-      <c r="E40" t="inlineStr"/>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>absolute_coefficient</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>history_of_heart_failure</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>LogisticRegression</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>categorical__BMI,kg/m2 (IMC)_26-30 kg/m2</t>
-        </is>
-      </c>
-      <c r="D41" t="n">
-        <v>0.6005183110480256</v>
-      </c>
-      <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>absolute_coefficient</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>history_of_heart_failure</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>LogisticRegression</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>categorical__Temperature_Higher</t>
-        </is>
-      </c>
-      <c r="D42" t="n">
-        <v>0.5159555265778009</v>
-      </c>
-      <c r="E42" t="inlineStr"/>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>absolute_coefficient</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>history_of_heart_failure</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>LogisticRegression</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>categorical__Blood pressure_Stage1</t>
-        </is>
-      </c>
-      <c r="D43" t="n">
-        <v>0.5124349512056834</v>
-      </c>
-      <c r="E43" t="inlineStr"/>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>absolute_coefficient</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>history_of_heart_failure</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>LogisticRegression</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>categorical__Blood pressure_Elevate</t>
-        </is>
-      </c>
-      <c r="D44" t="n">
-        <v>0.488674090173021</v>
-      </c>
-      <c r="E44" t="inlineStr"/>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>absolute_coefficient</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>history_of_heart_failure</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>LogisticRegression</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>categorical__Heart Rate_95</t>
-        </is>
-      </c>
-      <c r="D45" t="n">
-        <v>0.4876245236845273</v>
-      </c>
-      <c r="E45" t="inlineStr"/>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>absolute_coefficient</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>history_of_heart_failure</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>LogisticRegression</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>categorical__Location_Pasto</t>
-        </is>
-      </c>
-      <c r="D46" t="n">
-        <v>0.4576314581670638</v>
-      </c>
-      <c r="E46" t="inlineStr"/>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>absolute_coefficient</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>history_of_heart_failure</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>LogisticRegression</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>categorical__Sputum_Purulento</t>
-        </is>
-      </c>
-      <c r="D47" t="n">
-        <v>0.4443652264026181</v>
-      </c>
-      <c r="E47" t="inlineStr"/>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>absolute_coefficient</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>history_of_heart_failure</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>LogisticRegression</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>categorical__Heart Rate_74</t>
-        </is>
-      </c>
-      <c r="D48" t="n">
-        <v>0.4119957074582567</v>
-      </c>
-      <c r="E48" t="inlineStr"/>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>absolute_coefficient</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>history_of_heart_failure</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>LogisticRegression</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>categorical__BMI,kg/m2 (IMC)_21&lt;BMI&lt;25</t>
-        </is>
-      </c>
-      <c r="D49" t="n">
-        <v>0.4113048590893124</v>
-      </c>
-      <c r="E49" t="inlineStr"/>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>absolute_coefficient</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>history_of_heart_failure</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>LogisticRegression</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>categorical__Sputum_Purlent</t>
-        </is>
-      </c>
-      <c r="D50" t="n">
-        <v>0.4092281088618338</v>
-      </c>
-      <c r="E50" t="inlineStr"/>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>absolute_coefficient</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>history_of_heart_failure</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>LogisticRegression</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>categorical__BMI,kg/m2 (IMC)_≥35 kg/m2</t>
-        </is>
-      </c>
-      <c r="D51" t="n">
-        <v>0.4075715510438426</v>
-      </c>
-      <c r="E51" t="inlineStr"/>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>absolute_coefficient</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>history_of_heart_failure</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>LogisticRegression</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>categorical__Genero Sexo_Hombre</t>
-        </is>
-      </c>
-      <c r="D52" t="n">
-        <v>0.4005440423962965</v>
-      </c>
-      <c r="E52" t="inlineStr"/>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>absolute_coefficient</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>history_of_heart_failure</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>LogisticRegression</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>categorical__Genero Sexo_Mujer</t>
-        </is>
-      </c>
-      <c r="D53" t="n">
-        <v>0.3996570771141933</v>
-      </c>
-      <c r="E53" t="inlineStr"/>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>absolute_coefficient</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>history_of_heart_failure</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>LogisticRegression</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>categorical__Heart Rate_117</t>
-        </is>
-      </c>
-      <c r="D54" t="n">
-        <v>0.3986449161368875</v>
-      </c>
-      <c r="E54" t="inlineStr"/>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>absolute_coefficient</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>history_of_heart_failure</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>LogisticRegression</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>categorical__BMI,kg/m2 (IMC)_25≥ BMI &lt;30</t>
-        </is>
-      </c>
-      <c r="D55" t="n">
-        <v>0.3974827929690864</v>
-      </c>
-      <c r="E55" t="inlineStr"/>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>absolute_coefficient</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>history_of_heart_failure</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>LogisticRegression</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>categorical__Location_Cali</t>
-        </is>
-      </c>
-      <c r="D56" t="n">
-        <v>0.3782152754945572</v>
-      </c>
-      <c r="E56" t="inlineStr"/>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>absolute_coefficient</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>history_of_heart_failure</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>LogisticRegression</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>categorical__Heart Rate_67</t>
-        </is>
-      </c>
-      <c r="D57" t="n">
-        <v>0.3748122796227184</v>
-      </c>
-      <c r="E57" t="inlineStr"/>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>absolute_coefficient</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>history_of_heart_failure</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>LogisticRegression</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>categorical__status of smoking_Activo</t>
-        </is>
-      </c>
-      <c r="D58" t="n">
-        <v>0.3709584466524421</v>
-      </c>
-      <c r="E58" t="inlineStr"/>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>absolute_coefficient</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>history_of_heart_failure</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>LogisticRegression</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>categorical__Heart Rate_Higher</t>
-        </is>
-      </c>
-      <c r="D59" t="n">
-        <v>0.3709321680734826</v>
-      </c>
-      <c r="E59" t="inlineStr"/>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>absolute_coefficient</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>history_of_heart_failure</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>LogisticRegression</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>categorical__Heart Rate_86</t>
-        </is>
-      </c>
-      <c r="D60" t="n">
-        <v>0.3610485040919504</v>
-      </c>
-      <c r="E60" t="inlineStr"/>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>absolute_coefficient</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>history_of_heart_failure</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>LogisticRegression</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>categorical__Heart Rate_79</t>
-        </is>
-      </c>
-      <c r="D61" t="n">
-        <v>0.3506909526074221</v>
-      </c>
-      <c r="E61" t="inlineStr"/>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>absolute_coefficient</t>
+          <t>error: Pipeline should either be a classifier to be used with response_method=predict_proba or the response_method should be 'predict'. Got a regressor with response_method=predict_proba instead.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F61"/>
+  <autoFilter ref="A1:F32"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4943,10 +4245,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
     <col width="48" customWidth="1" min="2" max="2"/>
     <col width="48" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
@@ -4989,117 +4291,61 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>bodex</t>
+          <t>escala_disnea</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>BODEX (0 a 10 puntos) (Target)</t>
+          <t>ESCALA DISNEA (0 a 10 puntos) (Target)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>existe una sola clase observada; no es posible entrenar un clasificador | faltan clases del dominio teórico: 0, 1, 2, 3, 5, 6, 7, 8, 9, 10 | cobertura del dominio=9.09% &lt; 100.00%</t>
+          <t>faltan clases del dominio teórico: 0, 1, 3, 5, 6, 7, 8, 9 | cobertura del dominio=27.27% &lt; 100.00% | clases con representación insuficiente: 4=3</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>360</v>
+        <v>269</v>
       </c>
       <c r="E2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>{"0": 0, "1": 0, "2": 0, "3": 0, "4": 360, "5": 0, "6": 0, "7": 0, "8": 0, "9": 0, "10": 0}</t>
+          <t>{"0": 0, "1": 0, "2": 8, "3": 0, "4": 3, "5": 0, "6": 0, "7": 0, "8": 0, "9": 0, "10": 258}</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>escala_disnea</t>
+          <t>clasifisui</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ESCALA DISNEA (0 a 10 puntos) (Target)</t>
+          <t>CLASIFISUI (1 a 5, clasificacion urgencias) (Target)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>faltan clases del dominio teórico: 0, 1, 3, 5, 6, 7, 8, 9 | cobertura del dominio=27.27% &lt; 100.00% | clases con representación insuficiente: 4=3</t>
+          <t>faltan clases del dominio teórico: 1, 2, 3 | cobertura del dominio=40.00% &lt; 100.00%</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>360</v>
+        <v>269</v>
       </c>
       <c r="E3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>{"0": 0, "1": 0, "2": 8, "3": 0, "4": 3, "5": 0, "6": 0, "7": 0, "8": 0, "9": 0, "10": 349}</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>epocconfirmadosi_o_no_target</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>EPOCCONFIRMADO(Si ó no) (Target)</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>no existe un dominio teórico configurado para este target</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>456</v>
-      </c>
-      <c r="E4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>{"1": 456}</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>clasifisui</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>CLASIFISUI (1 a 5, clasificacion urgencias) (Target)</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>faltan clases del dominio teórico: 1, 2, 3 | cobertura del dominio=40.00% &lt; 100.00%</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>360</v>
-      </c>
-      <c r="E5" t="n">
-        <v>2</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>{"1": 0, "2": 0, "3": 0, "4": 58, "5": 302}</t>
+          <t>{"1": 0, "2": 0, "3": 0, "4": 47, "5": 222}</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F5"/>
+  <autoFilter ref="A1:F3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5115,13 +4361,13 @@
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="39" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
     <col width="23" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
     <col width="19" customWidth="1" min="10" max="10"/>
     <col width="26" customWidth="1" min="11" max="11"/>
     <col width="48" customWidth="1" min="12" max="12"/>
@@ -5250,7 +4496,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -5259,29 +4505,29 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="F3" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>0.4375</v>
+        <v>0.4857142857142858</v>
       </c>
       <c r="J3" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>55.98958333333333</v>
+        <v>32.11309523809524</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>ml\outputs\SavedModels\history_of_heart_failure-logisticregression.joblib</t>
+          <t>ml\outputs\SavedModels\history_of_heart_failure-catboost.joblib</t>
         </is>
       </c>
     </row>
@@ -6758,7 +6004,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>NOMBRE_DIAG</t>
+          <t>PESO</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -6768,7 +6014,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Diagnóstico registrado en la fuente clínica.</t>
+          <t>Peso corporal en la unidad registrada.</t>
         </is>
       </c>
     </row>
@@ -6785,7 +6031,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>PESO</t>
+          <t>TALLA(altura ó Height/m)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -6795,7 +6041,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Peso corporal en la unidad registrada.</t>
+          <t>Estatura del paciente; se conserva como predictor.</t>
         </is>
       </c>
     </row>
@@ -6812,7 +6058,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>TALLA(altura ó Height/m)</t>
+          <t>DISCAPACIDAD</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -6822,7 +6068,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Estatura del paciente; se conserva como predictor.</t>
+          <t>Indicador de discapacidad registrado.</t>
         </is>
       </c>
     </row>
@@ -6839,7 +6085,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>DISCAPACIDAD</t>
+          <t>TIPODISCAPAC</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -6849,7 +6095,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Indicador de discapacidad registrado.</t>
+          <t>Tipo de discapacidad registrada.</t>
         </is>
       </c>
     </row>
@@ -6866,7 +6112,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>TIPODISCAPAC</t>
+          <t>OCUPACION</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -6876,7 +6122,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Tipo de discapacidad registrada.</t>
+          <t>Ocupación registrada del paciente.</t>
         </is>
       </c>
     </row>
@@ -6893,7 +6139,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>OCUPACION</t>
+          <t>Altura_MSNM</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -6903,7 +6149,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Ocupación registrada del paciente.</t>
+          <t>Altitud del lugar de atención/localización en metros sobre el nivel del mar.</t>
         </is>
       </c>
     </row>
@@ -6920,7 +6166,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Altura_MSNM</t>
+          <t>Location</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -6930,7 +6176,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Altitud del lugar de atención/localización en metros sobre el nivel del mar.</t>
+          <t>Ubicación geográfica registrada.</t>
         </is>
       </c>
     </row>
@@ -6947,7 +6193,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Location</t>
+          <t>RIESGO CARDIOVASCULAR</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -6957,7 +6203,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Ubicación geográfica registrada.</t>
+          <t>Variable predictora disponible en el dataset; revisar definición de origen.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fastFix creacion de pacientes y informacion importante
</commit_message>
<xml_diff>
--- a/ml/outputs/SavedModels/training_metrics_report.xlsx
+++ b/ml/outputs/SavedModels/training_metrics_report.xlsx
@@ -12,26 +12,24 @@
     <sheet name="Hiperparametros" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Variables_Relevantes" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Tiempos_Prediccion" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Targets_Omitidos" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Resumen" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="CV_Detallado" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Variables_Seleccionadas" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Distribucion_Targets" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Graficos" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Metadatos" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Resumen" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="CV_Detallado" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Variables_Seleccionadas" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Distribucion_Targets" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Graficos" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Metadatos" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Comparacion_Modelos'!$A$1:$AN$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Particion_Datos'!$A$1:$K$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Hiperparametros'!$A$1:$E$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Variables_Relevantes'!$A$1:$F$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Variables_Relevantes'!$A$1:$F$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tiempos_Prediccion'!$A$1:$F$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Targets_Omitidos'!$A$1:$F$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Resumen'!$A$1:$L$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'CV_Detallado'!$A$1:$P$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Variables_Seleccionadas'!$A$1:$E$57</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Distribucion_Targets'!$A$1:$E$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Metadatos'!$A$1:$B$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Resumen'!$A$1:$L$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'CV_Detallado'!$A$1:$P$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Variables_Seleccionadas'!$A$1:$E$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Distribucion_Targets'!$A$1:$E$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Metadatos'!$A$1:$B$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2274,223 +2272,36 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:A4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="39" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>target</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>targetLabel</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>clase</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>porcentaje</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>copd_gold</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>COPD GOLD (1–4)</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>5</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0.3333333333333333</v>
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Artefactos gráficos</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>copd_gold</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>COPD GOLD (1–4)</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>5</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0.3333333333333333</v>
+          <t>Los gráficos detallados por target se exportan como PNG en Model_Reports/&lt;target&gt;/.</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>copd_gold</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>COPD GOLD (1–4)</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>3</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>copd_gold</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>COPD GOLD (1–4)</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>2</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0.1333333333333333</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>history_of_heart_failure</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Antecedente de insuficiencia cardiaca</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>7</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0.5833333333333334</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>history_of_heart_failure</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Antecedente de insuficiencia cardiaca</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>5</v>
-      </c>
-      <c r="E7" t="n">
-        <v>0.4166666666666667</v>
+          <t>Incluyen ROC comparativa, matrices de confusión, métricas, latencia y curvas de aprendizaje cuando corresponda.</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Artefactos gráficos</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Los gráficos detallados por target se exportan como PNG en Model_Reports/&lt;target&gt;/.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Incluyen ROC comparativa, matrices de confusión, métricas, latencia y curvas de aprendizaje cuando corresponda.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2547,7 +2358,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>{"accuracy": 0.7, "f1": 0.7, "mcc": 0.4, "kappa": 0.4, "auc": 0.7}</t>
+          <t>{"copd_gold": {"accuracy": 0.7, "f1": 0.7, "mcc": 0.4, "kappa": 0.4, "auc": 0.7, "modelQuality": 0.75}, "history_of_heart_failure": {"accuracy": 0.7, "f1": 0.7, "mcc": 0.4, "kappa": 0.4, "auc": 0.7, "modelQuality": 0.7}}</t>
         </is>
       </c>
     </row>
@@ -3273,15 +3084,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="19" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="48" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4156,30 +3967,8 @@
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>history_of_heart_failure</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>CatBoost</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>No disponible</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>error: Pipeline should either be a classifier to be used with response_method=predict_proba or the response_method should be 'predict'. Got a regressor with response_method=predict_proba instead.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:F32"/>
+  <autoFilter ref="A1:F31"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4240,117 +4029,6 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="48" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>target</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>column</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>reason</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>validRows</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>classes</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>classDistribution</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>escala_disnea</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>ESCALA DISNEA (0 a 10 puntos) (Target)</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>faltan clases del dominio teórico: 0, 1, 3, 5, 6, 7, 8, 9 | cobertura del dominio=27.27% &lt; 100.00% | clases con representación insuficiente: 4=3</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>269</v>
-      </c>
-      <c r="E2" t="n">
-        <v>3</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>{"0": 0, "1": 0, "2": 8, "3": 0, "4": 3, "5": 0, "6": 0, "7": 0, "8": 0, "9": 0, "10": 258}</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>clasifisui</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>CLASIFISUI (1 a 5, clasificacion urgencias) (Target)</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>faltan clases del dominio teórico: 1, 2, 3 | cobertura del dominio=40.00% &lt; 100.00%</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>269</v>
-      </c>
-      <c r="E3" t="n">
-        <v>2</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>{"1": 0, "2": 0, "3": 0, "4": 47, "5": 222}</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:F3"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4537,7 +4215,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4652,7 +4330,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6211,4 +5889,191 @@
   <autoFilter ref="A1:E57"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="39" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>targetLabel</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>clase</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>porcentaje</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>copd_gold</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>COPD GOLD (1–4)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>copd_gold</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>COPD GOLD (1–4)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>copd_gold</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>COPD GOLD (1–4)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>copd_gold</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>COPD GOLD (1–4)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.1333333333333333</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>history_of_heart_failure</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Antecedente de insuficiencia cardiaca</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>7</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>history_of_heart_failure</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Antecedente de insuficiencia cardiaca</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>5</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E7"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
actualizacion, necesidad de revisar GOLD 1 a 4
</commit_message>
<xml_diff>
--- a/ml/outputs/SavedModels/training_metrics_report.xlsx
+++ b/ml/outputs/SavedModels/training_metrics_report.xlsx
@@ -720,7 +720,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -916,7 +916,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -1700,7 +1700,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>{"copd_gold": {"accuracy": 0.7, "f1": 0.7, "mcc": 0.4, "kappa": 0.4, "auc": 0.7, "modelQuality": 0.75}, "history_of_heart_failure": {"accuracy": 0.7, "f1": 0.7, "mcc": 0.4, "kappa": 0.4, "auc": 0.7, "modelQuality": 0.7}}</t>
+          <t>{"copd_gold": {"accuracy": 0.7, "f1": 0.7, "mcc": 0.4, "kappa": 0.4, "auc": 0.7}, "history_of_heart_failure": {"accuracy": 0.7, "f1": 0.7, "mcc": 0.4, "kappa": 0.4, "auc": 0.7}}</t>
         </is>
       </c>
     </row>
@@ -4042,11 +4042,11 @@
     <col width="19" customWidth="1" min="3" max="3"/>
     <col width="23" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="21" customWidth="1" min="9" max="9"/>
-    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
     <col width="26" customWidth="1" min="11" max="11"/>
     <col width="48" customWidth="1" min="12" max="12"/>
   </cols>
@@ -4126,7 +4126,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -4135,29 +4135,29 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.8666666666666667</v>
+        <v>0.7333333333333333</v>
       </c>
       <c r="F2" t="n">
-        <v>0.9285714285714286</v>
+        <v>0.7</v>
       </c>
       <c r="G2" t="n">
-        <v>0.9</v>
+        <v>0.7333333333333334</v>
       </c>
       <c r="H2" t="n">
-        <v>0.8958333333333334</v>
+        <v>0.6888888888888889</v>
       </c>
       <c r="I2" t="n">
-        <v>0.99</v>
+        <v>0.8776068376068377</v>
       </c>
       <c r="J2" t="n">
-        <v>0.835710894037345</v>
+        <v>0.6503189868852074</v>
       </c>
       <c r="K2" t="n">
-        <v>91.32917853746886</v>
+        <v>76.38665410465082</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>ml\outputs\SavedModels\copd_gold-xgboost.joblib</t>
+          <t>ml\outputs\SavedModels\copd_gold-catboost.joblib</t>
         </is>
       </c>
     </row>
@@ -4172,42 +4172,13 @@
           <t>Antecedente de insuficiencia cardiaca</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>CatBoost</t>
-        </is>
-      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="E3" t="n">
-        <v>0.5833333333333334</v>
-      </c>
-      <c r="F3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0.4857142857142858</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="n">
-        <v>32.11309523809524</v>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>ml\outputs\SavedModels\history_of_heart_failure-catboost.joblib</t>
-        </is>
-      </c>
+      <c r="L3" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:L3"/>

</xml_diff>

<commit_message>
actualizacion generar todas las imagenes de calidad
</commit_message>
<xml_diff>
--- a/ml/outputs/SavedModels/training_metrics_report.xlsx
+++ b/ml/outputs/SavedModels/training_metrics_report.xlsx
@@ -27,7 +27,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tiempos_Prediccion'!$A$1:$F$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Resumen'!$A$1:$L$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'CV_Detallado'!$A$1:$P$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Variables_Seleccionadas'!$A$1:$E$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Variables_Seleccionadas'!$A$1:$E$63</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Distribucion_Targets'!$A$1:$E$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Metadatos'!$A$1:$B$9</definedName>
   </definedNames>
@@ -457,13 +457,13 @@
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="21" customWidth="1" min="8" max="8"/>
     <col width="21" customWidth="1" min="9" max="9"/>
-    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
     <col width="21" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
     <col width="21" customWidth="1" min="13" max="13"/>
     <col width="21" customWidth="1" min="14" max="14"/>
     <col width="20" customWidth="1" min="15" max="15"/>
-    <col width="21" customWidth="1" min="16" max="16"/>
+    <col width="22" customWidth="1" min="16" max="16"/>
     <col width="22" customWidth="1" min="17" max="17"/>
     <col width="21" customWidth="1" min="18" max="18"/>
     <col width="26" customWidth="1" min="19" max="19"/>
@@ -725,41 +725,41 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>0.6981796410006491</v>
+        <v>0.8500668838883184</v>
       </c>
       <c r="I2" t="n">
-        <v>0.7218428110993059</v>
+        <v>0.4115821721312407</v>
       </c>
       <c r="J2" t="n">
-        <v>0.05531678862705329</v>
+        <v>0.01579449780108281</v>
       </c>
       <c r="K2" t="n">
-        <v>0.6875</v>
+        <v>0.8875</v>
       </c>
       <c r="L2" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.8571428571428571</v>
       </c>
       <c r="M2" t="n">
-        <v>0.7083333333333333</v>
+        <v>0.8541666666666666</v>
       </c>
       <c r="N2" t="n">
-        <v>0.6892857142857143</v>
+        <v>0.8507936507936508</v>
       </c>
       <c r="O2" t="n">
-        <v>0.9022727272727273</v>
+        <v>0.9348484848484848</v>
       </c>
       <c r="P2" t="n">
-        <v>0.620704416451776</v>
+        <v>0.8195234918033747</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.6164383561643836</v>
+        <v>0.8082191780821918</v>
       </c>
       <c r="R2" t="n">
-        <v>0.7083333333333333</v>
+        <v>0.8541666666666666</v>
       </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr"/>
@@ -780,7 +780,7 @@
       <c r="AI2" t="inlineStr"/>
       <c r="AJ2" t="inlineStr"/>
       <c r="AK2" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="AL2" t="n">
         <v>14</v>
@@ -827,37 +827,37 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>0.4587347149150859</v>
+        <v>0.1556070494634678</v>
       </c>
       <c r="I3" t="n">
-        <v>0.3373921080737929</v>
+        <v>0.2350231053365259</v>
       </c>
       <c r="J3" t="n">
-        <v>0.09337965042254821</v>
+        <v>0.03885705293159283</v>
       </c>
       <c r="K3" t="n">
-        <v>0.4583333333333333</v>
+        <v>0.175</v>
       </c>
       <c r="L3" t="n">
-        <v>0.5</v>
+        <v>0.2142857142857143</v>
       </c>
       <c r="M3" t="n">
-        <v>0.4791666666666666</v>
+        <v>0.2083333333333333</v>
       </c>
       <c r="N3" t="n">
-        <v>0.4595238095238094</v>
+        <v>0.189484126984127</v>
       </c>
       <c r="O3" t="n">
-        <v>0.7270833333333333</v>
+        <v>0.5200757575757575</v>
       </c>
       <c r="P3" t="n">
-        <v>0.3311173112565667</v>
+        <v>-0.06340544258104468</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.3241379310344827</v>
+        <v>-0.06206896551724128</v>
       </c>
       <c r="R3" t="n">
-        <v>0.4791666666666666</v>
+        <v>0.2083333333333333</v>
       </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr"/>
@@ -878,7 +878,7 @@
       <c r="AI3" t="inlineStr"/>
       <c r="AJ3" t="inlineStr"/>
       <c r="AK3" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="AL3" t="n">
         <v>14</v>
@@ -916,46 +916,46 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
       <c r="H4" t="n">
-        <v>0.7818678099135439</v>
+        <v>0.85345703540347</v>
       </c>
       <c r="I4" t="n">
-        <v>0.6610063270859833</v>
+        <v>0.6027497901740975</v>
       </c>
       <c r="J4" t="n">
-        <v>0.08991087054204888</v>
+        <v>0.1100342151834005</v>
       </c>
       <c r="K4" t="n">
-        <v>0.8375</v>
+        <v>0.8875</v>
       </c>
       <c r="L4" t="n">
-        <v>0.7857142857142857</v>
+        <v>0.8571428571428571</v>
       </c>
       <c r="M4" t="n">
-        <v>0.7916666666666666</v>
+        <v>0.8541666666666666</v>
       </c>
       <c r="N4" t="n">
-        <v>0.8041666666666667</v>
+        <v>0.8507936507936508</v>
       </c>
       <c r="O4" t="n">
-        <v>0.9170454545454545</v>
+        <v>0.96875</v>
       </c>
       <c r="P4" t="n">
-        <v>0.7153467767436237</v>
+        <v>0.8195234918033747</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.710344827586207</v>
+        <v>0.8082191780821918</v>
       </c>
       <c r="R4" t="n">
-        <v>0.7916666666666666</v>
+        <v>0.8541666666666666</v>
       </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr"/>
@@ -976,7 +976,7 @@
       <c r="AI4" t="inlineStr"/>
       <c r="AJ4" t="inlineStr"/>
       <c r="AK4" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="AL4" t="n">
         <v>14</v>
@@ -1023,37 +1023,37 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>0.765833407166251</v>
+        <v>0.8494418838883184</v>
       </c>
       <c r="I5" t="n">
-        <v>0.7660041561011978</v>
+        <v>0.5436962099737888</v>
       </c>
       <c r="J5" t="n">
-        <v>0.123166892445981</v>
+        <v>0.06011531841385837</v>
       </c>
       <c r="K5" t="n">
+        <v>0.8875</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.8571428571428571</v>
+      </c>
+      <c r="M5" t="n">
         <v>0.8541666666666666</v>
       </c>
-      <c r="L5" t="n">
-        <v>0.7857142857142857</v>
-      </c>
-      <c r="M5" t="n">
-        <v>0.7708333333333334</v>
-      </c>
       <c r="N5" t="n">
-        <v>0.7535714285714286</v>
+        <v>0.8507936507936508</v>
       </c>
       <c r="O5" t="n">
-        <v>0.8679924242424242</v>
+        <v>0.9285984848484848</v>
       </c>
       <c r="P5" t="n">
-        <v>0.7363908738684537</v>
+        <v>0.8195234918033747</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.710344827586207</v>
+        <v>0.8082191780821918</v>
       </c>
       <c r="R5" t="n">
-        <v>0.7708333333333334</v>
+        <v>0.8541666666666666</v>
       </c>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr"/>
@@ -1074,7 +1074,7 @@
       <c r="AI5" t="inlineStr"/>
       <c r="AJ5" t="inlineStr"/>
       <c r="AK5" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="AL5" t="n">
         <v>14</v>
@@ -1112,46 +1112,46 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>0.697485619489256</v>
+        <v>0.8540820354034699</v>
       </c>
       <c r="I6" t="n">
-        <v>0.7844813451002542</v>
+        <v>0.7158847833438595</v>
       </c>
       <c r="J6" t="n">
-        <v>0.09665484830832617</v>
+        <v>0.04720807037516574</v>
       </c>
       <c r="K6" t="n">
-        <v>0.7125</v>
+        <v>0.8875</v>
       </c>
       <c r="L6" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.8571428571428571</v>
       </c>
       <c r="M6" t="n">
-        <v>0.7083333333333333</v>
+        <v>0.8541666666666666</v>
       </c>
       <c r="N6" t="n">
-        <v>0.6952380952380952</v>
+        <v>0.8507936507936508</v>
       </c>
       <c r="O6" t="n">
-        <v>0.8768939393939394</v>
+        <v>0.975</v>
       </c>
       <c r="P6" t="n">
-        <v>0.6250602903585061</v>
+        <v>0.8195234918033747</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.6164383561643836</v>
+        <v>0.8082191780821918</v>
       </c>
       <c r="R6" t="n">
-        <v>0.7083333333333333</v>
+        <v>0.8541666666666666</v>
       </c>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr"/>
@@ -1172,7 +1172,7 @@
       <c r="AI6" t="inlineStr"/>
       <c r="AJ6" t="inlineStr"/>
       <c r="AK6" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="AL6" t="n">
         <v>14</v>
@@ -1215,41 +1215,41 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>0.6952507710044076</v>
+        <v>0.7887133513336382</v>
       </c>
       <c r="I7" t="n">
-        <v>0.4876148990953708</v>
+        <v>0.3089127050464724</v>
       </c>
       <c r="J7" t="n">
-        <v>0.09148832674172856</v>
+        <v>0.03468036757288508</v>
       </c>
       <c r="K7" t="n">
-        <v>0.7125</v>
+        <v>0.8928571428571428</v>
       </c>
       <c r="L7" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.7857142857142857</v>
       </c>
       <c r="M7" t="n">
-        <v>0.7083333333333333</v>
+        <v>0.8125</v>
       </c>
       <c r="N7" t="n">
-        <v>0.6952380952380952</v>
+        <v>0.7818181818181819</v>
       </c>
       <c r="O7" t="n">
-        <v>0.8545454545454546</v>
+        <v>0.9174242424242424</v>
       </c>
       <c r="P7" t="n">
-        <v>0.6250602903585061</v>
+        <v>0.7607674567748487</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.6164383561643836</v>
+        <v>0.7123287671232876</v>
       </c>
       <c r="R7" t="n">
-        <v>0.7083333333333333</v>
+        <v>0.8125</v>
       </c>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr"/>
@@ -1270,7 +1270,7 @@
       <c r="AI7" t="inlineStr"/>
       <c r="AJ7" t="inlineStr"/>
       <c r="AK7" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="AL7" t="n">
         <v>14</v>
@@ -1317,37 +1317,37 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>0.4630659384038094</v>
+        <v>0.4758587837125155</v>
       </c>
       <c r="I8" t="n">
-        <v>0.4298335287550849</v>
+        <v>0.3299050364926633</v>
       </c>
       <c r="J8" t="n">
-        <v>0.1437952014675728</v>
+        <v>0.0752653091113273</v>
       </c>
       <c r="K8" t="n">
-        <v>0.5166666666666666</v>
+        <v>0.35</v>
       </c>
       <c r="L8" t="n">
         <v>0.5</v>
       </c>
       <c r="M8" t="n">
-        <v>0.4791666666666666</v>
+        <v>0.5</v>
       </c>
       <c r="N8" t="n">
-        <v>0.492063492063492</v>
+        <v>0.4083333333333333</v>
       </c>
       <c r="O8" t="n">
-        <v>0.6984848484848485</v>
+        <v>0.8821969696969698</v>
       </c>
       <c r="P8" t="n">
-        <v>0.3310423554409472</v>
+        <v>0.3686449626698406</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.3287671232876712</v>
+        <v>0.3378378378378379</v>
       </c>
       <c r="R8" t="n">
-        <v>0.4791666666666666</v>
+        <v>0.5</v>
       </c>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr"/>
@@ -1368,7 +1368,7 @@
       <c r="AI8" t="inlineStr"/>
       <c r="AJ8" t="inlineStr"/>
       <c r="AK8" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="AL8" t="n">
         <v>14</v>
@@ -1415,37 +1415,37 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>0.6078522056552473</v>
+        <v>0.4736681181837383</v>
       </c>
       <c r="I9" t="n">
-        <v>0.3892946234036278</v>
+        <v>0.3512016675592242</v>
       </c>
       <c r="J9" t="n">
-        <v>0.1297625288014696</v>
+        <v>0.03964606668919689</v>
       </c>
       <c r="K9" t="n">
-        <v>0.5625</v>
+        <v>0.3678571428571429</v>
       </c>
       <c r="L9" t="n">
-        <v>0.6428571428571429</v>
+        <v>0.5</v>
       </c>
       <c r="M9" t="n">
-        <v>0.625</v>
+        <v>0.5</v>
       </c>
       <c r="N9" t="n">
-        <v>0.5785714285714285</v>
+        <v>0.4068181818181819</v>
       </c>
       <c r="O9" t="n">
-        <v>0.8054924242424242</v>
+        <v>0.8630681818181818</v>
       </c>
       <c r="P9" t="n">
-        <v>0.5362069469915925</v>
+        <v>0.3733177575885583</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.5172413793103449</v>
+        <v>0.3333333333333334</v>
       </c>
       <c r="R9" t="n">
-        <v>0.625</v>
+        <v>0.5</v>
       </c>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr"/>
@@ -1466,7 +1466,7 @@
       <c r="AI9" t="inlineStr"/>
       <c r="AJ9" t="inlineStr"/>
       <c r="AK9" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="AL9" t="n">
         <v>14</v>
@@ -2369,7 +2369,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="6">
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D2" t="n">
         <v>14</v>
@@ -2522,13 +2522,13 @@
         <v>15</v>
       </c>
       <c r="F2" t="n">
-        <v>69.47368421052632</v>
+        <v>69.79166666666666</v>
       </c>
       <c r="G2" t="n">
-        <v>14.73684210526316</v>
+        <v>14.58333333333333</v>
       </c>
       <c r="H2" t="n">
-        <v>15.78947368421053</v>
+        <v>15.625</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -3088,8 +3088,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="48" customWidth="1" min="6" max="6"/>
@@ -3135,7 +3135,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CatBoost</t>
+          <t>ExtraTrees</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -3144,10 +3144,10 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.4666666666666666</v>
+        <v>0.4888888888888889</v>
       </c>
       <c r="E2" t="n">
-        <v>0.09428090415820629</v>
+        <v>0.0628539361054709</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3163,19 +3163,19 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CatBoost</t>
+          <t>ExtraTrees</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Location</t>
+          <t>BMI,kg/m2 (IMC)</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.0666666666666666</v>
+        <v>0.0444444444444444</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0544331053951817</v>
+        <v>0.0314269680527354</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -3191,19 +3191,19 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CatBoost</t>
+          <t>ExtraTrees</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>PackHistory</t>
+          <t>status of smoking</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>0.0222222222222222</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>0.0314269680527354</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -3219,19 +3219,19 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CatBoost</t>
+          <t>ExtraTrees</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>MWT1Best</t>
+          <t>Temperature</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>0.0222222222222222</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>0.0314269680527354</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -3247,19 +3247,19 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CatBoost</t>
+          <t>ExtraTrees</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>MWT1</t>
+          <t>Location</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>0.0222222222222222</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>0.0314269680527354</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -3275,12 +3275,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CatBoost</t>
+          <t>ExtraTrees</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>FVC</t>
+          <t>PackHistory</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -3303,7 +3303,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CatBoost</t>
+          <t>ExtraTrees</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -3331,12 +3331,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CatBoost</t>
+          <t>ExtraTrees</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>HAD</t>
+          <t>MWT1Best</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -3359,12 +3359,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CatBoost</t>
+          <t>ExtraTrees</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>smoking</t>
+          <t>FEV1PRED</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -3387,7 +3387,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CatBoost</t>
+          <t>ExtraTrees</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -3415,12 +3415,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CatBoost</t>
+          <t>ExtraTrees</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>CAT</t>
+          <t>FVC</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -3443,12 +3443,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CatBoost</t>
+          <t>ExtraTrees</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Respiratory Rate</t>
+          <t>CAT</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -3471,12 +3471,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CatBoost</t>
+          <t>ExtraTrees</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Heart Rate</t>
+          <t>MWT1</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -3499,12 +3499,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CatBoost</t>
+          <t>ExtraTrees</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>mMRC</t>
+          <t>MWT2</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -3527,12 +3527,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CatBoost</t>
+          <t>ExtraTrees</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>FEV1PRED</t>
+          <t>EDAD</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -3555,12 +3555,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>CatBoost</t>
+          <t>ExtraTrees</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>OCUPACION</t>
+          <t>smoking</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -3583,12 +3583,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CatBoost</t>
+          <t>ExtraTrees</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Altura_MSNM</t>
+          <t>SGRQ</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -3611,12 +3611,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>CatBoost</t>
+          <t>ExtraTrees</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>PESO</t>
+          <t>HAD</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -3639,12 +3639,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CatBoost</t>
+          <t>ExtraTrees</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>AtrialFib</t>
+          <t>mMRC</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -3667,12 +3667,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CatBoost</t>
+          <t>ExtraTrees</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>DISCAPACIDAD</t>
+          <t>AtrialFib</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -3695,12 +3695,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CatBoost</t>
+          <t>ExtraTrees</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>TIPODISCAPAC</t>
+          <t>TALLA(altura ó Height/m)</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -3723,19 +3723,19 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CatBoost</t>
+          <t>ExtraTrees</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>MWT2</t>
+          <t>Respiratory Rate</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>-0.0222222222222222</v>
+        <v>0</v>
       </c>
       <c r="E23" t="n">
-        <v>0.0314269680527354</v>
+        <v>0</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -3751,19 +3751,19 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CatBoost</t>
+          <t>ExtraTrees</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>SGRQ</t>
+          <t>Oxygen Saturation</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>-0.0222222222222222</v>
+        <v>0</v>
       </c>
       <c r="E24" t="n">
-        <v>0.0314269680527354</v>
+        <v>0</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -3779,19 +3779,19 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CatBoost</t>
+          <t>ExtraTrees</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Oxygen Saturation</t>
+          <t>DISCAPACIDAD</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>-0.0222222222222222</v>
+        <v>0</v>
       </c>
       <c r="E25" t="n">
-        <v>0.0314269680527354</v>
+        <v>0</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -3807,19 +3807,19 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CatBoost</t>
+          <t>ExtraTrees</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Temperature</t>
+          <t>TIPODISCAPAC</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>-0.0222222222222222</v>
+        <v>0</v>
       </c>
       <c r="E26" t="n">
-        <v>0.0314269680527354</v>
+        <v>0</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -3835,19 +3835,19 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CatBoost</t>
+          <t>ExtraTrees</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Blood pressure</t>
+          <t>OCUPACION</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>-0.0222222222222222</v>
+        <v>0</v>
       </c>
       <c r="E27" t="n">
-        <v>0.0314269680527354</v>
+        <v>0</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -3863,19 +3863,19 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CatBoost</t>
+          <t>ExtraTrees</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>EDAD</t>
+          <t>PESO</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>-0.0444444444444445</v>
+        <v>0</v>
       </c>
       <c r="E28" t="n">
-        <v>0.0314269680527354</v>
+        <v>0</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -3891,19 +3891,19 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CatBoost</t>
+          <t>ExtraTrees</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>status of smoking</t>
+          <t>Altura_MSNM</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>-0.0444444444444445</v>
+        <v>0</v>
       </c>
       <c r="E29" t="n">
-        <v>0.0314269680527354</v>
+        <v>0</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -3919,7 +3919,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CatBoost</t>
+          <t>ExtraTrees</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -3928,7 +3928,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>-0.0444444444444445</v>
+        <v>-0.0222222222222222</v>
       </c>
       <c r="E30" t="n">
         <v>0.0314269680527354</v>
@@ -3947,16 +3947,16 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CatBoost</t>
+          <t>ExtraTrees</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>BMI,kg/m2 (IMC)</t>
+          <t>Heart Rate</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>-0.0444444444444445</v>
+        <v>-0.0222222222222222</v>
       </c>
       <c r="E31" t="n">
         <v>0.0314269680527354</v>
@@ -4148,7 +4148,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>CatBoost</t>
+          <t>ExtraTrees</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -4157,29 +4157,29 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.7333333333333333</v>
+        <v>0.8666666666666667</v>
       </c>
       <c r="F2" t="n">
-        <v>0.7</v>
+        <v>0.875</v>
       </c>
       <c r="G2" t="n">
-        <v>0.7333333333333334</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="H2" t="n">
-        <v>0.6888888888888889</v>
+        <v>0.8022727272727272</v>
       </c>
       <c r="I2" t="n">
-        <v>0.8776068376068377</v>
+        <v>0.9549358974358975</v>
       </c>
       <c r="J2" t="n">
-        <v>0.6503189868852074</v>
+        <v>0.8293797509006984</v>
       </c>
       <c r="K2" t="n">
-        <v>76.38665410465082</v>
+        <v>87.33830164536191</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>ml\outputs\SavedModels\copd_gold-catboost.joblib</t>
+          <t>ml\outputs\SavedModels\copd_gold-extratrees.joblib</t>
         </is>
       </c>
     </row>
@@ -4358,7 +4358,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E57"/>
+  <dimension ref="A1:E63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -5893,22 +5893,184 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
+          <t>Glucose</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>seleccionado_por_target</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Variable predictora disponible en el dataset; revisar definición de origen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>history_of_heart_failure</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Antecedente de insuficiencia cardiaca</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Creatinine</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>seleccionado_por_target</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Variable predictora disponible en el dataset; revisar definición de origen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>history_of_heart_failure</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Antecedente de insuficiencia cardiaca</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>BNP</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>seleccionado_por_target</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Variable predictora disponible en el dataset; revisar definición de origen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>history_of_heart_failure</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Antecedente de insuficiencia cardiaca</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>ECG</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>seleccionado_por_target</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Variable predictora disponible en el dataset; revisar definición de origen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>history_of_heart_failure</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Antecedente de insuficiencia cardiaca</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Coronary History</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>seleccionado_por_target</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Variable predictora disponible en el dataset; revisar definición de origen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>history_of_heart_failure</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Antecedente de insuficiencia cardiaca</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Arrhythmias</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>seleccionado_por_target</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Variable predictora disponible en el dataset; revisar definición de origen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>history_of_heart_failure</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Antecedente de insuficiencia cardiaca</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
           <t>RIESGO CARDIOVASCULAR</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr">
+      <c r="D63" t="inlineStr">
         <is>
           <t>seleccionado_por_target</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr">
+      <c r="E63" t="inlineStr">
         <is>
           <t>Variable predictora disponible en el dataset; revisar definición de origen.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E57"/>
+  <autoFilter ref="A1:E63"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>